<commit_message>
Update: describe your changes
</commit_message>
<xml_diff>
--- a/docs/bulk-send/bulk-review-requests-sample.xlsx
+++ b/docs/bulk-send/bulk-review-requests-sample.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/johntang/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/johntang/Desktop/clients/baam-review/docs/bulk-send/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E456C4D7-1FAF-6E4D-B992-D49ADB645A8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90DFAD1B-D0AC-9241-89D4-3A88EF2AE81B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Customers" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
   <si>
     <t>Name</t>
   </si>
@@ -103,15 +103,6 @@
     <t>phone only — SMS preferred</t>
   </si>
   <si>
-    <t>Patrick O'Connor</t>
-  </si>
-  <si>
-    <t>patrick.o@example.com</t>
-  </si>
-  <si>
-    <t>(212) 555-0179</t>
-  </si>
-  <si>
     <t>john.tang2025@gmail.com</t>
   </si>
   <si>
@@ -119,6 +110,21 @@
   </si>
   <si>
     <t>support@baamplatform.com</t>
+  </si>
+  <si>
+    <t>Company</t>
+  </si>
+  <si>
+    <t>Primary care center</t>
+  </si>
+  <si>
+    <t>TCM Center</t>
+  </si>
+  <si>
+    <t>Acupuncture Land</t>
+  </si>
+  <si>
+    <t>Taco Paradise</t>
   </si>
 </sst>
 </file>
@@ -506,145 +512,140 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="32.83203125" customWidth="1"/>
+    <col min="1" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="28.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="5" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="32.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>31</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" t="s">
         <v>7</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>8</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>9</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>32</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D3" t="s">
         <v>12</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>13</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>14</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>16</v>
       </c>
       <c r="B4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C4" t="s">
         <v>17</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>18</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>19</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>20</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="B5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" t="s">
         <v>23</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>24</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>25</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>26</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B6" t="s">
-        <v>28</v>
-      </c>
-      <c r="C6" t="s">
-        <v>29</v>
-      </c>
-      <c r="D6" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" t="s">
-        <v>25</v>
-      </c>
-      <c r="F6" t="s">
-        <v>18</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B5" r:id="rId1" xr:uid="{AF127563-488A-FC4B-9338-08D1997BE4BE}"/>
-    <hyperlink ref="B2" r:id="rId2" xr:uid="{3B300326-3579-074B-A54E-198556495991}"/>
-    <hyperlink ref="B3" r:id="rId3" xr:uid="{CD44F59B-D922-5948-AEBD-97A14F61A05A}"/>
+    <hyperlink ref="C5" r:id="rId1" xr:uid="{AF127563-488A-FC4B-9338-08D1997BE4BE}"/>
+    <hyperlink ref="C2" r:id="rId2" xr:uid="{3B300326-3579-074B-A54E-198556495991}"/>
+    <hyperlink ref="C3" r:id="rId3" xr:uid="{CD44F59B-D922-5948-AEBD-97A14F61A05A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:F1 A6:F6 A5 C5:F5 A4:F4 A2 C2:F2 A3 C3:F3" numberStoredAsText="1"/>
+    <ignoredError sqref="C1:G1 D5:G5 C4:G4 D2:G3 A1:A5" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>